<commit_message>
fix(utaustin): enable dual openpyxl cell.hyperlink objects and sanitize pipe-separated DOI formulas in Excel workbook
</commit_message>
<xml_diff>
--- a/universities_wise/ut_austin/ut_austin_aerospace_mechanical_faculty.xlsx
+++ b/universities_wise/ut_austin/ut_austin_aerospace_mechanical_faculty.xlsx
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="X2" s="3">
-        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2607.28976 | https://doi.org/10.1063/5.0325672", "https://doi.org/10.48550/arxiv.2607.28976 | https://doi.org/10.1063/5.0325672")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2607.28976", "https://doi.org/10.48550/arxiv.2607.28976 | https://doi.org/10.1063/5.0325672")</f>
         <v/>
       </c>
       <c r="Y2" s="2" t="inlineStr">
@@ -1032,7 +1032,7 @@
         </is>
       </c>
       <c r="X3" s="3">
-        <f>HYPERLINK("https://doi.org/10.1080/13647830.2026.2621925 | https://doi.org/10.48550/arxiv.2607.25048", "https://doi.org/10.1080/13647830.2026.2621925 | https://doi.org/10.48550/arxiv.2607.25048")</f>
+        <f>HYPERLINK("https://doi.org/10.1080/13647830.2026.2621925", "https://doi.org/10.1080/13647830.2026.2621925 | https://doi.org/10.48550/arxiv.2607.25048")</f>
         <v/>
       </c>
       <c r="Y3" s="2" t="inlineStr">
@@ -1205,7 +1205,7 @@
         </is>
       </c>
       <c r="X4" s="3">
-        <f>HYPERLINK("https://doi.org/10.2514/6.2026-0460 | https://doi.org/10.2514/6.2026-1315", "https://doi.org/10.2514/6.2026-0460 | https://doi.org/10.2514/6.2026-1315")</f>
+        <f>HYPERLINK("https://doi.org/10.2514/6.2026-0460", "https://doi.org/10.2514/6.2026-0460 | https://doi.org/10.2514/6.2026-1315")</f>
         <v/>
       </c>
       <c r="Y4" s="2" t="inlineStr">
@@ -1374,7 +1374,7 @@
         </is>
       </c>
       <c r="X5" s="3">
-        <f>HYPERLINK("https://doi.org/10.2514/6.2025-1302 | https://doi.org/10.2514/6.2025-1162", "https://doi.org/10.2514/6.2025-1302 | https://doi.org/10.2514/6.2025-1162")</f>
+        <f>HYPERLINK("https://doi.org/10.2514/6.2025-1302", "https://doi.org/10.2514/6.2025-1302 | https://doi.org/10.2514/6.2025-1162")</f>
         <v/>
       </c>
       <c r="Y5" s="2" t="inlineStr">
@@ -1543,7 +1543,7 @@
         </is>
       </c>
       <c r="X6" s="3">
-        <f>HYPERLINK("https://doi.org/10.1029/2025jh000697 | https://doi.org/10.24433/co.5021363.v1", "https://doi.org/10.1029/2025jh000697 | https://doi.org/10.24433/co.5021363.v1")</f>
+        <f>HYPERLINK("https://doi.org/10.1029/2025jh000697", "https://doi.org/10.1029/2025jh000697 | https://doi.org/10.24433/co.5021363.v1")</f>
         <v/>
       </c>
       <c r="Y6" s="2" t="inlineStr">
@@ -1716,7 +1716,7 @@
         </is>
       </c>
       <c r="X7" s="3">
-        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2604.03158 | https://doi.org/10.48550/arxiv.2603.24189", "https://doi.org/10.48550/arxiv.2604.03158 | https://doi.org/10.48550/arxiv.2603.24189")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2604.03158", "https://doi.org/10.48550/arxiv.2604.03158 | https://doi.org/10.48550/arxiv.2603.24189")</f>
         <v/>
       </c>
       <c r="Y7" s="2" t="inlineStr">
@@ -1889,7 +1889,7 @@
         </is>
       </c>
       <c r="X8" s="3">
-        <f>HYPERLINK("https://doi.org/10.1029/2025je009389 | https://doi.org/10.48550/arxiv.2607.23904", "https://doi.org/10.1029/2025je009389 | https://doi.org/10.48550/arxiv.2607.23904")</f>
+        <f>HYPERLINK("https://doi.org/10.1029/2025je009389", "https://doi.org/10.1029/2025je009389 | https://doi.org/10.48550/arxiv.2607.23904")</f>
         <v/>
       </c>
       <c r="Y8" s="2" t="inlineStr">
@@ -2058,7 +2058,7 @@
         </is>
       </c>
       <c r="X9" s="3">
-        <f>HYPERLINK("https://doi.org/10.1016/j.cma.2026.119046 | https://doi.org/10.1142/s021820252650003x", "https://doi.org/10.1016/j.cma.2026.119046 | https://doi.org/10.1142/s021820252650003x")</f>
+        <f>HYPERLINK("https://doi.org/10.1016/j.cma.2026.119046", "https://doi.org/10.1016/j.cma.2026.119046 | https://doi.org/10.1142/s021820252650003x")</f>
         <v/>
       </c>
       <c r="Y9" s="2" t="inlineStr">
@@ -2231,7 +2231,7 @@
         </is>
       </c>
       <c r="X10" s="3">
-        <f>HYPERLINK("https://doi.org/10.1115/1.4069945 | https://doi.org/10.1115/1.4069942", "https://doi.org/10.1115/1.4069945 | https://doi.org/10.1115/1.4069942")</f>
+        <f>HYPERLINK("https://doi.org/10.1115/1.4069945", "https://doi.org/10.1115/1.4069945 | https://doi.org/10.1115/1.4069942")</f>
         <v/>
       </c>
       <c r="Y10" s="2" t="inlineStr">
@@ -2512,7 +2512,7 @@
         </is>
       </c>
       <c r="X12" s="3">
-        <f>HYPERLINK("https://doi.org/10.1007/s10444-026-10322-7 | https://doi.org/10.1186/s12911-026-03520-2", "https://doi.org/10.1007/s10444-026-10322-7 | https://doi.org/10.1186/s12911-026-03520-2")</f>
+        <f>HYPERLINK("https://doi.org/10.1007/s10444-026-10322-7", "https://doi.org/10.1007/s10444-026-10322-7 | https://doi.org/10.1186/s12911-026-03520-2")</f>
         <v/>
       </c>
       <c r="Y12" s="2" t="inlineStr">
@@ -2801,7 +2801,7 @@
         </is>
       </c>
       <c r="X14" s="3">
-        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2502.16555 | https://doi.org/10.1088/1361-6595/ae0c33", "https://doi.org/10.48550/arxiv.2502.16555 | https://doi.org/10.1088/1361-6595/ae0c33")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2502.16555", "https://doi.org/10.48550/arxiv.2502.16555 | https://doi.org/10.1088/1361-6595/ae0c33")</f>
         <v/>
       </c>
       <c r="Y14" s="2" t="inlineStr">
@@ -2978,7 +2978,7 @@
         </is>
       </c>
       <c r="X15" s="3">
-        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2608.02223 | https://doi.org/10.48550/arxiv.2607.28932", "https://doi.org/10.48550/arxiv.2608.02223 | https://doi.org/10.48550/arxiv.2607.28932")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2608.02223", "https://doi.org/10.48550/arxiv.2608.02223 | https://doi.org/10.48550/arxiv.2607.28932")</f>
         <v/>
       </c>
       <c r="Y15" s="2" t="inlineStr">
@@ -3155,7 +3155,7 @@
         </is>
       </c>
       <c r="X16" s="3">
-        <f>HYPERLINK("https://doi.org/10.2514/1.b40460 | https://doi.org/10.1063/5.0325672", "https://doi.org/10.2514/1.b40460 | https://doi.org/10.1063/5.0325672")</f>
+        <f>HYPERLINK("https://doi.org/10.2514/1.b40460", "https://doi.org/10.2514/1.b40460 | https://doi.org/10.1063/5.0325672")</f>
         <v/>
       </c>
       <c r="Y16" s="2" t="inlineStr">
@@ -3332,7 +3332,7 @@
         </is>
       </c>
       <c r="X17" s="3">
-        <f>HYPERLINK("https://doi.org/10.1115/es2025-155214 | https://doi.org/10.1126/sciadv.aed5744", "https://doi.org/10.1115/es2025-155214 | https://doi.org/10.1126/sciadv.aed5744")</f>
+        <f>HYPERLINK("https://doi.org/10.1115/es2025-155214", "https://doi.org/10.1115/es2025-155214 | https://doi.org/10.1126/sciadv.aed5744")</f>
         <v/>
       </c>
       <c r="Y17" s="2" t="inlineStr">
@@ -3509,7 +3509,7 @@
         </is>
       </c>
       <c r="X18" s="3">
-        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2609.07912 | https://doi.org/10.1137/25m1753097", "https://doi.org/10.48550/arxiv.2609.07912 | https://doi.org/10.1137/25m1753097")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2609.07912", "https://doi.org/10.48550/arxiv.2609.07912 | https://doi.org/10.1137/25m1753097")</f>
         <v/>
       </c>
       <c r="Y18" s="2" t="inlineStr">
@@ -3798,7 +3798,7 @@
         </is>
       </c>
       <c r="X20" s="3">
-        <f>HYPERLINK("https://doi.org/10.1002/aenm.71193 | https://doi.org/10.6084/m9.figshare.32570274", "https://doi.org/10.1002/aenm.71193 | https://doi.org/10.6084/m9.figshare.32570274")</f>
+        <f>HYPERLINK("https://doi.org/10.1002/aenm.71193", "https://doi.org/10.1002/aenm.71193 | https://doi.org/10.6084/m9.figshare.32570274")</f>
         <v/>
       </c>
       <c r="Y20" s="2" t="inlineStr">
@@ -3975,7 +3975,7 @@
         </is>
       </c>
       <c r="X21" s="3">
-        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2602.22097 | https://doi.org/10.1137/24m1668755", "https://doi.org/10.48550/arxiv.2602.22097 | https://doi.org/10.1137/24m1668755")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2602.22097", "https://doi.org/10.48550/arxiv.2602.22097 | https://doi.org/10.1137/24m1668755")</f>
         <v/>
       </c>
       <c r="Y21" s="2" t="inlineStr">
@@ -4148,7 +4148,7 @@
         </is>
       </c>
       <c r="X22" s="3">
-        <f>HYPERLINK("https://doi.org/10.1137/25m1737341 | https://doi.org/10.1007/978-3-032-00094-1_66", "https://doi.org/10.1137/25m1737341 | https://doi.org/10.1007/978-3-032-00094-1_66")</f>
+        <f>HYPERLINK("https://doi.org/10.1137/25m1737341", "https://doi.org/10.1137/25m1737341 | https://doi.org/10.1007/978-3-032-00094-1_66")</f>
         <v/>
       </c>
       <c r="Y22" s="2" t="inlineStr">
@@ -4321,7 +4321,7 @@
         </is>
       </c>
       <c r="X23" s="3">
-        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2603.03211 | https://doi.org/10.2514/6.2026-1210", "https://doi.org/10.48550/arxiv.2603.03211 | https://doi.org/10.2514/6.2026-1210")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2603.03211", "https://doi.org/10.48550/arxiv.2603.03211 | https://doi.org/10.2514/6.2026-1210")</f>
         <v/>
       </c>
       <c r="Y23" s="2" t="inlineStr">
@@ -4494,7 +4494,7 @@
         </is>
       </c>
       <c r="X24" s="3">
-        <f>HYPERLINK("https://doi.org/10.1137/25m175857x | https://doi.org/10.1137/24m1678027", "https://doi.org/10.1137/25m175857x | https://doi.org/10.1137/24m1678027")</f>
+        <f>HYPERLINK("https://doi.org/10.1137/25m175857x", "https://doi.org/10.1137/25m175857x | https://doi.org/10.1137/24m1678027")</f>
         <v/>
       </c>
       <c r="Y24" s="2" t="inlineStr">
@@ -4667,7 +4667,7 @@
         </is>
       </c>
       <c r="X25" s="3">
-        <f>HYPERLINK("https://doi.org/10.5802/smai-jcm.132 | https://doi.org/10.1038/s41467-025-65681-4", "https://doi.org/10.5802/smai-jcm.132 | https://doi.org/10.1038/s41467-025-65681-4")</f>
+        <f>HYPERLINK("https://doi.org/10.5802/smai-jcm.132", "https://doi.org/10.5802/smai-jcm.132 | https://doi.org/10.1038/s41467-025-65681-4")</f>
         <v/>
       </c>
       <c r="Y25" s="2" t="inlineStr">
@@ -4840,7 +4840,7 @@
         </is>
       </c>
       <c r="X26" s="3">
-        <f>HYPERLINK("https://doi.org/10.1007/s10915-025-02938-6 | https://doi.org/10.1201/9781003492139-1", "https://doi.org/10.1007/s10915-025-02938-6 | https://doi.org/10.1201/9781003492139-1")</f>
+        <f>HYPERLINK("https://doi.org/10.1007/s10915-025-02938-6", "https://doi.org/10.1007/s10915-025-02938-6 | https://doi.org/10.1201/9781003492139-1")</f>
         <v/>
       </c>
       <c r="Y26" s="2" t="inlineStr">
@@ -5013,7 +5013,7 @@
         </is>
       </c>
       <c r="X27" s="3">
-        <f>HYPERLINK("https://doi.org/10.4208/jiasc.2026-91-1 | https://doi.org/10.4171/ifb/547", "https://doi.org/10.4208/jiasc.2026-91-1 | https://doi.org/10.4171/ifb/547")</f>
+        <f>HYPERLINK("https://doi.org/10.4208/jiasc.2026-91-1", "https://doi.org/10.4208/jiasc.2026-91-1 | https://doi.org/10.4171/ifb/547")</f>
         <v/>
       </c>
       <c r="Y27" s="2" t="inlineStr">
@@ -5083,6 +5083,181 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P2" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T2" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X2" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV2" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P3" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T3" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X3" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV3" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P4" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T4" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X4" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV4" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P5" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T5" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X5" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV5" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P6" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T6" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X6" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV6" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P7" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T7" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X7" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV7" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P8" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T8" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X8" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV8" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P9" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T9" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X9" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV9" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P10" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T10" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X10" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV10" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV11" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P12" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T12" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X12" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV12" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV13" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P14" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T14" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X14" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV14" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P15" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T15" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X15" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV15" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P16" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T16" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X16" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV16" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P17" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T17" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X17" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV17" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P18" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T18" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X18" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV18" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV19" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P20" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T20" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X20" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV20" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P21" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T21" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X21" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV21" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P22" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T22" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X22" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV22" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P23" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T23" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X23" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV23" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P24" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T24" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X24" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV24" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P25" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T25" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X25" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV25" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P26" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T26" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X26" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV26" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P27" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T27" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X27" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV27" r:id="rId173"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5492,7 +5667,7 @@
         </is>
       </c>
       <c r="X2" s="3">
-        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2607.28976 | https://doi.org/10.1063/5.0325672", "https://doi.org/10.48550/arxiv.2607.28976 | https://doi.org/10.1063/5.0325672")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2607.28976", "https://doi.org/10.48550/arxiv.2607.28976 | https://doi.org/10.1063/5.0325672")</f>
         <v/>
       </c>
       <c r="Y2" s="2" t="inlineStr">
@@ -5665,7 +5840,7 @@
         </is>
       </c>
       <c r="X3" s="3">
-        <f>HYPERLINK("https://doi.org/10.1080/13647830.2026.2621925 | https://doi.org/10.48550/arxiv.2607.25048", "https://doi.org/10.1080/13647830.2026.2621925 | https://doi.org/10.48550/arxiv.2607.25048")</f>
+        <f>HYPERLINK("https://doi.org/10.1080/13647830.2026.2621925", "https://doi.org/10.1080/13647830.2026.2621925 | https://doi.org/10.48550/arxiv.2607.25048")</f>
         <v/>
       </c>
       <c r="Y3" s="2" t="inlineStr">
@@ -5838,7 +6013,7 @@
         </is>
       </c>
       <c r="X4" s="3">
-        <f>HYPERLINK("https://doi.org/10.2514/6.2026-0460 | https://doi.org/10.2514/6.2026-1315", "https://doi.org/10.2514/6.2026-0460 | https://doi.org/10.2514/6.2026-1315")</f>
+        <f>HYPERLINK("https://doi.org/10.2514/6.2026-0460", "https://doi.org/10.2514/6.2026-0460 | https://doi.org/10.2514/6.2026-1315")</f>
         <v/>
       </c>
       <c r="Y4" s="2" t="inlineStr">
@@ -6007,7 +6182,7 @@
         </is>
       </c>
       <c r="X5" s="3">
-        <f>HYPERLINK("https://doi.org/10.2514/6.2025-1302 | https://doi.org/10.2514/6.2025-1162", "https://doi.org/10.2514/6.2025-1302 | https://doi.org/10.2514/6.2025-1162")</f>
+        <f>HYPERLINK("https://doi.org/10.2514/6.2025-1302", "https://doi.org/10.2514/6.2025-1302 | https://doi.org/10.2514/6.2025-1162")</f>
         <v/>
       </c>
       <c r="Y5" s="2" t="inlineStr">
@@ -6176,7 +6351,7 @@
         </is>
       </c>
       <c r="X6" s="3">
-        <f>HYPERLINK("https://doi.org/10.1029/2025jh000697 | https://doi.org/10.24433/co.5021363.v1", "https://doi.org/10.1029/2025jh000697 | https://doi.org/10.24433/co.5021363.v1")</f>
+        <f>HYPERLINK("https://doi.org/10.1029/2025jh000697", "https://doi.org/10.1029/2025jh000697 | https://doi.org/10.24433/co.5021363.v1")</f>
         <v/>
       </c>
       <c r="Y6" s="2" t="inlineStr">
@@ -6349,7 +6524,7 @@
         </is>
       </c>
       <c r="X7" s="3">
-        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2604.03158 | https://doi.org/10.48550/arxiv.2603.24189", "https://doi.org/10.48550/arxiv.2604.03158 | https://doi.org/10.48550/arxiv.2603.24189")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2604.03158", "https://doi.org/10.48550/arxiv.2604.03158 | https://doi.org/10.48550/arxiv.2603.24189")</f>
         <v/>
       </c>
       <c r="Y7" s="2" t="inlineStr">
@@ -6522,7 +6697,7 @@
         </is>
       </c>
       <c r="X8" s="3">
-        <f>HYPERLINK("https://doi.org/10.1029/2025je009389 | https://doi.org/10.48550/arxiv.2607.23904", "https://doi.org/10.1029/2025je009389 | https://doi.org/10.48550/arxiv.2607.23904")</f>
+        <f>HYPERLINK("https://doi.org/10.1029/2025je009389", "https://doi.org/10.1029/2025je009389 | https://doi.org/10.48550/arxiv.2607.23904")</f>
         <v/>
       </c>
       <c r="Y8" s="2" t="inlineStr">
@@ -6691,7 +6866,7 @@
         </is>
       </c>
       <c r="X9" s="3">
-        <f>HYPERLINK("https://doi.org/10.1016/j.cma.2026.119046 | https://doi.org/10.1142/s021820252650003x", "https://doi.org/10.1016/j.cma.2026.119046 | https://doi.org/10.1142/s021820252650003x")</f>
+        <f>HYPERLINK("https://doi.org/10.1016/j.cma.2026.119046", "https://doi.org/10.1016/j.cma.2026.119046 | https://doi.org/10.1142/s021820252650003x")</f>
         <v/>
       </c>
       <c r="Y9" s="2" t="inlineStr">
@@ -6864,7 +7039,7 @@
         </is>
       </c>
       <c r="X10" s="3">
-        <f>HYPERLINK("https://doi.org/10.1115/1.4069945 | https://doi.org/10.1115/1.4069942", "https://doi.org/10.1115/1.4069945 | https://doi.org/10.1115/1.4069942")</f>
+        <f>HYPERLINK("https://doi.org/10.1115/1.4069945", "https://doi.org/10.1115/1.4069945 | https://doi.org/10.1115/1.4069942")</f>
         <v/>
       </c>
       <c r="Y10" s="2" t="inlineStr">
@@ -7145,7 +7320,7 @@
         </is>
       </c>
       <c r="X12" s="3">
-        <f>HYPERLINK("https://doi.org/10.1007/s10444-026-10322-7 | https://doi.org/10.1186/s12911-026-03520-2", "https://doi.org/10.1007/s10444-026-10322-7 | https://doi.org/10.1186/s12911-026-03520-2")</f>
+        <f>HYPERLINK("https://doi.org/10.1007/s10444-026-10322-7", "https://doi.org/10.1007/s10444-026-10322-7 | https://doi.org/10.1186/s12911-026-03520-2")</f>
         <v/>
       </c>
       <c r="Y12" s="2" t="inlineStr">
@@ -7434,7 +7609,7 @@
         </is>
       </c>
       <c r="X14" s="3">
-        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2502.16555 | https://doi.org/10.1088/1361-6595/ae0c33", "https://doi.org/10.48550/arxiv.2502.16555 | https://doi.org/10.1088/1361-6595/ae0c33")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2502.16555", "https://doi.org/10.48550/arxiv.2502.16555 | https://doi.org/10.1088/1361-6595/ae0c33")</f>
         <v/>
       </c>
       <c r="Y14" s="2" t="inlineStr">
@@ -7611,7 +7786,7 @@
         </is>
       </c>
       <c r="X15" s="3">
-        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2608.02223 | https://doi.org/10.48550/arxiv.2607.28932", "https://doi.org/10.48550/arxiv.2608.02223 | https://doi.org/10.48550/arxiv.2607.28932")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2608.02223", "https://doi.org/10.48550/arxiv.2608.02223 | https://doi.org/10.48550/arxiv.2607.28932")</f>
         <v/>
       </c>
       <c r="Y15" s="2" t="inlineStr">
@@ -7788,7 +7963,7 @@
         </is>
       </c>
       <c r="X16" s="3">
-        <f>HYPERLINK("https://doi.org/10.2514/1.b40460 | https://doi.org/10.1063/5.0325672", "https://doi.org/10.2514/1.b40460 | https://doi.org/10.1063/5.0325672")</f>
+        <f>HYPERLINK("https://doi.org/10.2514/1.b40460", "https://doi.org/10.2514/1.b40460 | https://doi.org/10.1063/5.0325672")</f>
         <v/>
       </c>
       <c r="Y16" s="2" t="inlineStr">
@@ -7965,7 +8140,7 @@
         </is>
       </c>
       <c r="X17" s="3">
-        <f>HYPERLINK("https://doi.org/10.1115/es2025-155214 | https://doi.org/10.1126/sciadv.aed5744", "https://doi.org/10.1115/es2025-155214 | https://doi.org/10.1126/sciadv.aed5744")</f>
+        <f>HYPERLINK("https://doi.org/10.1115/es2025-155214", "https://doi.org/10.1115/es2025-155214 | https://doi.org/10.1126/sciadv.aed5744")</f>
         <v/>
       </c>
       <c r="Y17" s="2" t="inlineStr">
@@ -8142,7 +8317,7 @@
         </is>
       </c>
       <c r="X18" s="3">
-        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2609.07912 | https://doi.org/10.1137/25m1753097", "https://doi.org/10.48550/arxiv.2609.07912 | https://doi.org/10.1137/25m1753097")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2609.07912", "https://doi.org/10.48550/arxiv.2609.07912 | https://doi.org/10.1137/25m1753097")</f>
         <v/>
       </c>
       <c r="Y18" s="2" t="inlineStr">
@@ -8431,7 +8606,7 @@
         </is>
       </c>
       <c r="X20" s="3">
-        <f>HYPERLINK("https://doi.org/10.1002/aenm.71193 | https://doi.org/10.6084/m9.figshare.32570274", "https://doi.org/10.1002/aenm.71193 | https://doi.org/10.6084/m9.figshare.32570274")</f>
+        <f>HYPERLINK("https://doi.org/10.1002/aenm.71193", "https://doi.org/10.1002/aenm.71193 | https://doi.org/10.6084/m9.figshare.32570274")</f>
         <v/>
       </c>
       <c r="Y20" s="2" t="inlineStr">
@@ -8608,7 +8783,7 @@
         </is>
       </c>
       <c r="X21" s="3">
-        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2602.22097 | https://doi.org/10.1137/24m1668755", "https://doi.org/10.48550/arxiv.2602.22097 | https://doi.org/10.1137/24m1668755")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2602.22097", "https://doi.org/10.48550/arxiv.2602.22097 | https://doi.org/10.1137/24m1668755")</f>
         <v/>
       </c>
       <c r="Y21" s="2" t="inlineStr">
@@ -17094,6 +17269,463 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P2" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T2" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X2" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV2" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P3" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T3" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X3" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV3" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P4" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T4" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X4" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV4" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P5" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T5" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X5" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV5" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P6" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T6" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X6" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV6" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P7" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T7" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X7" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV7" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P8" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T8" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X8" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV8" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P9" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T9" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X9" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV9" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P10" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T10" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X10" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV10" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV11" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P12" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T12" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X12" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV12" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV13" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P14" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T14" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X14" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV14" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P15" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T15" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X15" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV15" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P16" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T16" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X16" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV16" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P17" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T17" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X17" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV17" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P18" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T18" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X18" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV18" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV19" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P20" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T20" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X20" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV20" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P21" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T21" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X21" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV21" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV22" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV23" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV24" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV25" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV26" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV27" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV28" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV29" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV30" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV31" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV32" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV33" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV34" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV35" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D36" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV36" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV37" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D38" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV38" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV39" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV40" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV41" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D42" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV42" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D43" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV43" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C44" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D44" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV44" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C45" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D45" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV45" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C46" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D46" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H46" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV46" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C47" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D47" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H47" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV47" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C48" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D48" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H48" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV48" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C49" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D49" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H49" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV49" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D50" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H50" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV50" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C51" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D51" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H51" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV51" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C52" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D52" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H52" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV52" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C53" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D53" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H53" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV53" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C54" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D54" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H54" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV54" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C55" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D55" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H55" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV55" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C56" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D56" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H56" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV56" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C57" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D57" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H57" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV57" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C58" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D58" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H58" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV58" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C59" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D59" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV59" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C60" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D60" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H60" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV60" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C61" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D61" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H61" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV61" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C62" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D62" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H62" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV62" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C63" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D63" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H63" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV63" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C64" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D64" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H64" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV64" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C65" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D65" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H65" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV65" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C66" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D66" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H66" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV66" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C67" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D67" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H67" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV67" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C68" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D68" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H68" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV68" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C69" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D69" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H69" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV69" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C70" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D70" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H70" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV70" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C71" r:id="rId328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D71" r:id="rId329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H71" r:id="rId330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV71" r:id="rId331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C72" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D72" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H72" r:id="rId334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV72" r:id="rId335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C73" r:id="rId336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D73" r:id="rId337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H73" r:id="rId338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV73" r:id="rId339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C74" r:id="rId340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D74" r:id="rId341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H74" r:id="rId342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV74" r:id="rId343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C75" r:id="rId344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D75" r:id="rId345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H75" r:id="rId346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV75" r:id="rId347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C76" r:id="rId348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D76" r:id="rId349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H76" r:id="rId350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV76" r:id="rId351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C77" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D77" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H77" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV77" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C78" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D78" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H78" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV78" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C79" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D79" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H79" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV79" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C80" r:id="rId364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D80" r:id="rId365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H80" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV80" r:id="rId367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C81" r:id="rId368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D81" r:id="rId369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H81" r:id="rId370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV81" r:id="rId371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C82" r:id="rId372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D82" r:id="rId373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H82" r:id="rId374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV82" r:id="rId375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C83" r:id="rId376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D83" r:id="rId377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H83" r:id="rId378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV83" r:id="rId379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C84" r:id="rId380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D84" r:id="rId381"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H84" r:id="rId382"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV84" r:id="rId383"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C85" r:id="rId384"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D85" r:id="rId385"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H85" r:id="rId386"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV85" r:id="rId387"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C86" r:id="rId388"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D86" r:id="rId389"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H86" r:id="rId390"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV86" r:id="rId391"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C87" r:id="rId392"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D87" r:id="rId393"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H87" r:id="rId394"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV87" r:id="rId395"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C88" r:id="rId396"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D88" r:id="rId397"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H88" r:id="rId398"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV88" r:id="rId399"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C89" r:id="rId400"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D89" r:id="rId401"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H89" r:id="rId402"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV89" r:id="rId403"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C90" r:id="rId404"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D90" r:id="rId405"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H90" r:id="rId406"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV90" r:id="rId407"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C91" r:id="rId408"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D91" r:id="rId409"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H91" r:id="rId410"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV91" r:id="rId411"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C92" r:id="rId412"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D92" r:id="rId413"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H92" r:id="rId414"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV92" r:id="rId415"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C93" r:id="rId416"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D93" r:id="rId417"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H93" r:id="rId418"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV93" r:id="rId419"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C94" r:id="rId420"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D94" r:id="rId421"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H94" r:id="rId422"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV94" r:id="rId423"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C95" r:id="rId424"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D95" r:id="rId425"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H95" r:id="rId426"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV95" r:id="rId427"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C96" r:id="rId428"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D96" r:id="rId429"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H96" r:id="rId430"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV96" r:id="rId431"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C97" r:id="rId432"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D97" r:id="rId433"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H97" r:id="rId434"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV97" r:id="rId435"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C98" r:id="rId436"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D98" r:id="rId437"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H98" r:id="rId438"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV98" r:id="rId439"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C99" r:id="rId440"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D99" r:id="rId441"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H99" r:id="rId442"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV99" r:id="rId443"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C100" r:id="rId444"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D100" r:id="rId445"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H100" r:id="rId446"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV100" r:id="rId447"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C101" r:id="rId448"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D101" r:id="rId449"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H101" r:id="rId450"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV101" r:id="rId451"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C102" r:id="rId452"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D102" r:id="rId453"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H102" r:id="rId454"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV102" r:id="rId455"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17503,7 +18135,7 @@
         </is>
       </c>
       <c r="X2" s="3">
-        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2607.28976 | https://doi.org/10.1063/5.0325672", "https://doi.org/10.48550/arxiv.2607.28976 | https://doi.org/10.1063/5.0325672")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2607.28976", "https://doi.org/10.48550/arxiv.2607.28976 | https://doi.org/10.1063/5.0325672")</f>
         <v/>
       </c>
       <c r="Y2" s="2" t="inlineStr">
@@ -17676,7 +18308,7 @@
         </is>
       </c>
       <c r="X3" s="3">
-        <f>HYPERLINK("https://doi.org/10.1080/13647830.2026.2621925 | https://doi.org/10.48550/arxiv.2607.25048", "https://doi.org/10.1080/13647830.2026.2621925 | https://doi.org/10.48550/arxiv.2607.25048")</f>
+        <f>HYPERLINK("https://doi.org/10.1080/13647830.2026.2621925", "https://doi.org/10.1080/13647830.2026.2621925 | https://doi.org/10.48550/arxiv.2607.25048")</f>
         <v/>
       </c>
       <c r="Y3" s="2" t="inlineStr">
@@ -17849,7 +18481,7 @@
         </is>
       </c>
       <c r="X4" s="3">
-        <f>HYPERLINK("https://doi.org/10.2514/6.2026-0460 | https://doi.org/10.2514/6.2026-1315", "https://doi.org/10.2514/6.2026-0460 | https://doi.org/10.2514/6.2026-1315")</f>
+        <f>HYPERLINK("https://doi.org/10.2514/6.2026-0460", "https://doi.org/10.2514/6.2026-0460 | https://doi.org/10.2514/6.2026-1315")</f>
         <v/>
       </c>
       <c r="Y4" s="2" t="inlineStr">
@@ -18018,7 +18650,7 @@
         </is>
       </c>
       <c r="X5" s="3">
-        <f>HYPERLINK("https://doi.org/10.2514/6.2025-1302 | https://doi.org/10.2514/6.2025-1162", "https://doi.org/10.2514/6.2025-1302 | https://doi.org/10.2514/6.2025-1162")</f>
+        <f>HYPERLINK("https://doi.org/10.2514/6.2025-1302", "https://doi.org/10.2514/6.2025-1302 | https://doi.org/10.2514/6.2025-1162")</f>
         <v/>
       </c>
       <c r="Y5" s="2" t="inlineStr">
@@ -18187,7 +18819,7 @@
         </is>
       </c>
       <c r="X6" s="3">
-        <f>HYPERLINK("https://doi.org/10.1029/2025jh000697 | https://doi.org/10.24433/co.5021363.v1", "https://doi.org/10.1029/2025jh000697 | https://doi.org/10.24433/co.5021363.v1")</f>
+        <f>HYPERLINK("https://doi.org/10.1029/2025jh000697", "https://doi.org/10.1029/2025jh000697 | https://doi.org/10.24433/co.5021363.v1")</f>
         <v/>
       </c>
       <c r="Y6" s="2" t="inlineStr">
@@ -18360,7 +18992,7 @@
         </is>
       </c>
       <c r="X7" s="3">
-        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2604.03158 | https://doi.org/10.48550/arxiv.2603.24189", "https://doi.org/10.48550/arxiv.2604.03158 | https://doi.org/10.48550/arxiv.2603.24189")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2604.03158", "https://doi.org/10.48550/arxiv.2604.03158 | https://doi.org/10.48550/arxiv.2603.24189")</f>
         <v/>
       </c>
       <c r="Y7" s="2" t="inlineStr">
@@ -18533,7 +19165,7 @@
         </is>
       </c>
       <c r="X8" s="3">
-        <f>HYPERLINK("https://doi.org/10.1029/2025je009389 | https://doi.org/10.48550/arxiv.2607.23904", "https://doi.org/10.1029/2025je009389 | https://doi.org/10.48550/arxiv.2607.23904")</f>
+        <f>HYPERLINK("https://doi.org/10.1029/2025je009389", "https://doi.org/10.1029/2025je009389 | https://doi.org/10.48550/arxiv.2607.23904")</f>
         <v/>
       </c>
       <c r="Y8" s="2" t="inlineStr">
@@ -18702,7 +19334,7 @@
         </is>
       </c>
       <c r="X9" s="3">
-        <f>HYPERLINK("https://doi.org/10.1016/j.cma.2026.119046 | https://doi.org/10.1142/s021820252650003x", "https://doi.org/10.1016/j.cma.2026.119046 | https://doi.org/10.1142/s021820252650003x")</f>
+        <f>HYPERLINK("https://doi.org/10.1016/j.cma.2026.119046", "https://doi.org/10.1016/j.cma.2026.119046 | https://doi.org/10.1142/s021820252650003x")</f>
         <v/>
       </c>
       <c r="Y9" s="2" t="inlineStr">
@@ -18875,7 +19507,7 @@
         </is>
       </c>
       <c r="X10" s="3">
-        <f>HYPERLINK("https://doi.org/10.1115/1.4069945 | https://doi.org/10.1115/1.4069942", "https://doi.org/10.1115/1.4069945 | https://doi.org/10.1115/1.4069942")</f>
+        <f>HYPERLINK("https://doi.org/10.1115/1.4069945", "https://doi.org/10.1115/1.4069945 | https://doi.org/10.1115/1.4069942")</f>
         <v/>
       </c>
       <c r="Y10" s="2" t="inlineStr">
@@ -19156,7 +19788,7 @@
         </is>
       </c>
       <c r="X12" s="3">
-        <f>HYPERLINK("https://doi.org/10.1007/s10444-026-10322-7 | https://doi.org/10.1186/s12911-026-03520-2", "https://doi.org/10.1007/s10444-026-10322-7 | https://doi.org/10.1186/s12911-026-03520-2")</f>
+        <f>HYPERLINK("https://doi.org/10.1007/s10444-026-10322-7", "https://doi.org/10.1007/s10444-026-10322-7 | https://doi.org/10.1186/s12911-026-03520-2")</f>
         <v/>
       </c>
       <c r="Y12" s="2" t="inlineStr">
@@ -19445,7 +20077,7 @@
         </is>
       </c>
       <c r="X14" s="3">
-        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2502.16555 | https://doi.org/10.1088/1361-6595/ae0c33", "https://doi.org/10.48550/arxiv.2502.16555 | https://doi.org/10.1088/1361-6595/ae0c33")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2502.16555", "https://doi.org/10.48550/arxiv.2502.16555 | https://doi.org/10.1088/1361-6595/ae0c33")</f>
         <v/>
       </c>
       <c r="Y14" s="2" t="inlineStr">
@@ -19622,7 +20254,7 @@
         </is>
       </c>
       <c r="X15" s="3">
-        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2608.02223 | https://doi.org/10.48550/arxiv.2607.28932", "https://doi.org/10.48550/arxiv.2608.02223 | https://doi.org/10.48550/arxiv.2607.28932")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2608.02223", "https://doi.org/10.48550/arxiv.2608.02223 | https://doi.org/10.48550/arxiv.2607.28932")</f>
         <v/>
       </c>
       <c r="Y15" s="2" t="inlineStr">
@@ -19799,7 +20431,7 @@
         </is>
       </c>
       <c r="X16" s="3">
-        <f>HYPERLINK("https://doi.org/10.2514/1.b40460 | https://doi.org/10.1063/5.0325672", "https://doi.org/10.2514/1.b40460 | https://doi.org/10.1063/5.0325672")</f>
+        <f>HYPERLINK("https://doi.org/10.2514/1.b40460", "https://doi.org/10.2514/1.b40460 | https://doi.org/10.1063/5.0325672")</f>
         <v/>
       </c>
       <c r="Y16" s="2" t="inlineStr">
@@ -19976,7 +20608,7 @@
         </is>
       </c>
       <c r="X17" s="3">
-        <f>HYPERLINK("https://doi.org/10.1115/es2025-155214 | https://doi.org/10.1126/sciadv.aed5744", "https://doi.org/10.1115/es2025-155214 | https://doi.org/10.1126/sciadv.aed5744")</f>
+        <f>HYPERLINK("https://doi.org/10.1115/es2025-155214", "https://doi.org/10.1115/es2025-155214 | https://doi.org/10.1126/sciadv.aed5744")</f>
         <v/>
       </c>
       <c r="Y17" s="2" t="inlineStr">
@@ -20153,7 +20785,7 @@
         </is>
       </c>
       <c r="X18" s="3">
-        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2609.07912 | https://doi.org/10.1137/25m1753097", "https://doi.org/10.48550/arxiv.2609.07912 | https://doi.org/10.1137/25m1753097")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2609.07912", "https://doi.org/10.48550/arxiv.2609.07912 | https://doi.org/10.1137/25m1753097")</f>
         <v/>
       </c>
       <c r="Y18" s="2" t="inlineStr">
@@ -20442,7 +21074,7 @@
         </is>
       </c>
       <c r="X20" s="3">
-        <f>HYPERLINK("https://doi.org/10.1002/aenm.71193 | https://doi.org/10.6084/m9.figshare.32570274", "https://doi.org/10.1002/aenm.71193 | https://doi.org/10.6084/m9.figshare.32570274")</f>
+        <f>HYPERLINK("https://doi.org/10.1002/aenm.71193", "https://doi.org/10.1002/aenm.71193 | https://doi.org/10.6084/m9.figshare.32570274")</f>
         <v/>
       </c>
       <c r="Y20" s="2" t="inlineStr">
@@ -20619,7 +21251,7 @@
         </is>
       </c>
       <c r="X21" s="3">
-        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2602.22097 | https://doi.org/10.1137/24m1668755", "https://doi.org/10.48550/arxiv.2602.22097 | https://doi.org/10.1137/24m1668755")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2602.22097", "https://doi.org/10.48550/arxiv.2602.22097 | https://doi.org/10.1137/24m1668755")</f>
         <v/>
       </c>
       <c r="Y21" s="2" t="inlineStr">
@@ -20792,7 +21424,7 @@
         </is>
       </c>
       <c r="X22" s="3">
-        <f>HYPERLINK("https://doi.org/10.1137/25m1737341 | https://doi.org/10.1007/978-3-032-00094-1_66", "https://doi.org/10.1137/25m1737341 | https://doi.org/10.1007/978-3-032-00094-1_66")</f>
+        <f>HYPERLINK("https://doi.org/10.1137/25m1737341", "https://doi.org/10.1137/25m1737341 | https://doi.org/10.1007/978-3-032-00094-1_66")</f>
         <v/>
       </c>
       <c r="Y22" s="2" t="inlineStr">
@@ -20965,7 +21597,7 @@
         </is>
       </c>
       <c r="X23" s="3">
-        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2603.03211 | https://doi.org/10.2514/6.2026-1210", "https://doi.org/10.48550/arxiv.2603.03211 | https://doi.org/10.2514/6.2026-1210")</f>
+        <f>HYPERLINK("https://doi.org/10.48550/arxiv.2603.03211", "https://doi.org/10.48550/arxiv.2603.03211 | https://doi.org/10.2514/6.2026-1210")</f>
         <v/>
       </c>
       <c r="Y23" s="2" t="inlineStr">
@@ -21138,7 +21770,7 @@
         </is>
       </c>
       <c r="X24" s="3">
-        <f>HYPERLINK("https://doi.org/10.1137/25m175857x | https://doi.org/10.1137/24m1678027", "https://doi.org/10.1137/25m175857x | https://doi.org/10.1137/24m1678027")</f>
+        <f>HYPERLINK("https://doi.org/10.1137/25m175857x", "https://doi.org/10.1137/25m175857x | https://doi.org/10.1137/24m1678027")</f>
         <v/>
       </c>
       <c r="Y24" s="2" t="inlineStr">
@@ -21311,7 +21943,7 @@
         </is>
       </c>
       <c r="X25" s="3">
-        <f>HYPERLINK("https://doi.org/10.5802/smai-jcm.132 | https://doi.org/10.1038/s41467-025-65681-4", "https://doi.org/10.5802/smai-jcm.132 | https://doi.org/10.1038/s41467-025-65681-4")</f>
+        <f>HYPERLINK("https://doi.org/10.5802/smai-jcm.132", "https://doi.org/10.5802/smai-jcm.132 | https://doi.org/10.1038/s41467-025-65681-4")</f>
         <v/>
       </c>
       <c r="Y25" s="2" t="inlineStr">
@@ -21484,7 +22116,7 @@
         </is>
       </c>
       <c r="X26" s="3">
-        <f>HYPERLINK("https://doi.org/10.1007/s10915-025-02938-6 | https://doi.org/10.1201/9781003492139-1", "https://doi.org/10.1007/s10915-025-02938-6 | https://doi.org/10.1201/9781003492139-1")</f>
+        <f>HYPERLINK("https://doi.org/10.1007/s10915-025-02938-6", "https://doi.org/10.1007/s10915-025-02938-6 | https://doi.org/10.1201/9781003492139-1")</f>
         <v/>
       </c>
       <c r="Y26" s="2" t="inlineStr">
@@ -21657,7 +22289,7 @@
         </is>
       </c>
       <c r="X27" s="3">
-        <f>HYPERLINK("https://doi.org/10.4208/jiasc.2026-91-1 | https://doi.org/10.4171/ifb/547", "https://doi.org/10.4208/jiasc.2026-91-1 | https://doi.org/10.4171/ifb/547")</f>
+        <f>HYPERLINK("https://doi.org/10.4208/jiasc.2026-91-1", "https://doi.org/10.4208/jiasc.2026-91-1 | https://doi.org/10.4171/ifb/547")</f>
         <v/>
       </c>
       <c r="Y27" s="2" t="inlineStr">
@@ -37019,6 +37651,781 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P2" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T2" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X2" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV2" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P3" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T3" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X3" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV3" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P4" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T4" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X4" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV4" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P5" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T5" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X5" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV5" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P6" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T6" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X6" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV6" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P7" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T7" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X7" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV7" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P8" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T8" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X8" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV8" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P9" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T9" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X9" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV9" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P10" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T10" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X10" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV10" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV11" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P12" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T12" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X12" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV12" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV13" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P14" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T14" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X14" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV14" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P15" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T15" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X15" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV15" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P16" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T16" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X16" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV16" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P17" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T17" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X17" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV17" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P18" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T18" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X18" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV18" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV19" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P20" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T20" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X20" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV20" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P21" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T21" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X21" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV21" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P22" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T22" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X22" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV22" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P23" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T23" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X23" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV23" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P24" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T24" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X24" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV24" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P25" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T25" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X25" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV25" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P26" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T26" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X26" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV26" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P27" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T27" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X27" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV27" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV28" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV29" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV30" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV31" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV32" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV33" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV34" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV35" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D36" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV36" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV37" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D38" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV38" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV39" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV40" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV41" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D42" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV42" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D43" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV43" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C44" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D44" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV44" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C45" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D45" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV45" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C46" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D46" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H46" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV46" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C47" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D47" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H47" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV47" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C48" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D48" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H48" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV48" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C49" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D49" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H49" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV49" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D50" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H50" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV50" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C51" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D51" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H51" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV51" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C52" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D52" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H52" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV52" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C53" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D53" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H53" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV53" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C54" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D54" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H54" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV54" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C55" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D55" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H55" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV55" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C56" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D56" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H56" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV56" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C57" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D57" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H57" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV57" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C58" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D58" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H58" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV58" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C59" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D59" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV59" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C60" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D60" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H60" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV60" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C61" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D61" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H61" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV61" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C62" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D62" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H62" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV62" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C63" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D63" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H63" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV63" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C64" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D64" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H64" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV64" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C65" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D65" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H65" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV65" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C66" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D66" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H66" r:id="rId328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV66" r:id="rId329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C67" r:id="rId330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D67" r:id="rId331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H67" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV67" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C68" r:id="rId334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D68" r:id="rId335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H68" r:id="rId336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV68" r:id="rId337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C69" r:id="rId338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D69" r:id="rId339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H69" r:id="rId340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV69" r:id="rId341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C70" r:id="rId342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D70" r:id="rId343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H70" r:id="rId344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV70" r:id="rId345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C71" r:id="rId346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D71" r:id="rId347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H71" r:id="rId348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV71" r:id="rId349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C72" r:id="rId350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D72" r:id="rId351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H72" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV72" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C73" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D73" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H73" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV73" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C74" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D74" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H74" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV74" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C75" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D75" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H75" r:id="rId364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV75" r:id="rId365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C76" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D76" r:id="rId367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H76" r:id="rId368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV76" r:id="rId369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C77" r:id="rId370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D77" r:id="rId371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H77" r:id="rId372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV77" r:id="rId373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C78" r:id="rId374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D78" r:id="rId375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H78" r:id="rId376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV78" r:id="rId377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C79" r:id="rId378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D79" r:id="rId379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H79" r:id="rId380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV79" r:id="rId381"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C80" r:id="rId382"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D80" r:id="rId383"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H80" r:id="rId384"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV80" r:id="rId385"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C81" r:id="rId386"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D81" r:id="rId387"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H81" r:id="rId388"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV81" r:id="rId389"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C82" r:id="rId390"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D82" r:id="rId391"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H82" r:id="rId392"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV82" r:id="rId393"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C83" r:id="rId394"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D83" r:id="rId395"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H83" r:id="rId396"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV83" r:id="rId397"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C84" r:id="rId398"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D84" r:id="rId399"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H84" r:id="rId400"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV84" r:id="rId401"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C85" r:id="rId402"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D85" r:id="rId403"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H85" r:id="rId404"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV85" r:id="rId405"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C86" r:id="rId406"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D86" r:id="rId407"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H86" r:id="rId408"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV86" r:id="rId409"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C87" r:id="rId410"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D87" r:id="rId411"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H87" r:id="rId412"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV87" r:id="rId413"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C88" r:id="rId414"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D88" r:id="rId415"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H88" r:id="rId416"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV88" r:id="rId417"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C89" r:id="rId418"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D89" r:id="rId419"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H89" r:id="rId420"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV89" r:id="rId421"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C90" r:id="rId422"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D90" r:id="rId423"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H90" r:id="rId424"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV90" r:id="rId425"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C91" r:id="rId426"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D91" r:id="rId427"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H91" r:id="rId428"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV91" r:id="rId429"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C92" r:id="rId430"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D92" r:id="rId431"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H92" r:id="rId432"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV92" r:id="rId433"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C93" r:id="rId434"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D93" r:id="rId435"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H93" r:id="rId436"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV93" r:id="rId437"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C94" r:id="rId438"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D94" r:id="rId439"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H94" r:id="rId440"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV94" r:id="rId441"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C95" r:id="rId442"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D95" r:id="rId443"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H95" r:id="rId444"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV95" r:id="rId445"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C96" r:id="rId446"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D96" r:id="rId447"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H96" r:id="rId448"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV96" r:id="rId449"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C97" r:id="rId450"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D97" r:id="rId451"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H97" r:id="rId452"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV97" r:id="rId453"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C98" r:id="rId454"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D98" r:id="rId455"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H98" r:id="rId456"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV98" r:id="rId457"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C99" r:id="rId458"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D99" r:id="rId459"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H99" r:id="rId460"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV99" r:id="rId461"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C100" r:id="rId462"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D100" r:id="rId463"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H100" r:id="rId464"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV100" r:id="rId465"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C101" r:id="rId466"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D101" r:id="rId467"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H101" r:id="rId468"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV101" r:id="rId469"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C102" r:id="rId470"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D102" r:id="rId471"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H102" r:id="rId472"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV102" r:id="rId473"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C103" r:id="rId474"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D103" r:id="rId475"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H103" r:id="rId476"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV103" r:id="rId477"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C104" r:id="rId478"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D104" r:id="rId479"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H104" r:id="rId480"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV104" r:id="rId481"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C105" r:id="rId482"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D105" r:id="rId483"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H105" r:id="rId484"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV105" r:id="rId485"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C106" r:id="rId486"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D106" r:id="rId487"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H106" r:id="rId488"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV106" r:id="rId489"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C107" r:id="rId490"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D107" r:id="rId491"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H107" r:id="rId492"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV107" r:id="rId493"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C108" r:id="rId494"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D108" r:id="rId495"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H108" r:id="rId496"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV108" r:id="rId497"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C109" r:id="rId498"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D109" r:id="rId499"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H109" r:id="rId500"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV109" r:id="rId501"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C110" r:id="rId502"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D110" r:id="rId503"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H110" r:id="rId504"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV110" r:id="rId505"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C111" r:id="rId506"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D111" r:id="rId507"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H111" r:id="rId508"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV111" r:id="rId509"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C112" r:id="rId510"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D112" r:id="rId511"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H112" r:id="rId512"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV112" r:id="rId513"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C113" r:id="rId514"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D113" r:id="rId515"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H113" r:id="rId516"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV113" r:id="rId517"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C114" r:id="rId518"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D114" r:id="rId519"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H114" r:id="rId520"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV114" r:id="rId521"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C115" r:id="rId522"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D115" r:id="rId523"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H115" r:id="rId524"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV115" r:id="rId525"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C116" r:id="rId526"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D116" r:id="rId527"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H116" r:id="rId528"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV116" r:id="rId529"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C117" r:id="rId530"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D117" r:id="rId531"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H117" r:id="rId532"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV117" r:id="rId533"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C118" r:id="rId534"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D118" r:id="rId535"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H118" r:id="rId536"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV118" r:id="rId537"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C119" r:id="rId538"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D119" r:id="rId539"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H119" r:id="rId540"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV119" r:id="rId541"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C120" r:id="rId542"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D120" r:id="rId543"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H120" r:id="rId544"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV120" r:id="rId545"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C121" r:id="rId546"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D121" r:id="rId547"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H121" r:id="rId548"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV121" r:id="rId549"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C122" r:id="rId550"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D122" r:id="rId551"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H122" r:id="rId552"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV122" r:id="rId553"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C123" r:id="rId554"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D123" r:id="rId555"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H123" r:id="rId556"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV123" r:id="rId557"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C124" r:id="rId558"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D124" r:id="rId559"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H124" r:id="rId560"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV124" r:id="rId561"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C125" r:id="rId562"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D125" r:id="rId563"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H125" r:id="rId564"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV125" r:id="rId565"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C126" r:id="rId566"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D126" r:id="rId567"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H126" r:id="rId568"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV126" r:id="rId569"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C127" r:id="rId570"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D127" r:id="rId571"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H127" r:id="rId572"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV127" r:id="rId573"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C128" r:id="rId574"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D128" r:id="rId575"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H128" r:id="rId576"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV128" r:id="rId577"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C129" r:id="rId578"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D129" r:id="rId579"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H129" r:id="rId580"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV129" r:id="rId581"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C130" r:id="rId582"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D130" r:id="rId583"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H130" r:id="rId584"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV130" r:id="rId585"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C131" r:id="rId586"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D131" r:id="rId587"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H131" r:id="rId588"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV131" r:id="rId589"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C132" r:id="rId590"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D132" r:id="rId591"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H132" r:id="rId592"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV132" r:id="rId593"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C133" r:id="rId594"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D133" r:id="rId595"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H133" r:id="rId596"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV133" r:id="rId597"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C134" r:id="rId598"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D134" r:id="rId599"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H134" r:id="rId600"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV134" r:id="rId601"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C135" r:id="rId602"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D135" r:id="rId603"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H135" r:id="rId604"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV135" r:id="rId605"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C136" r:id="rId606"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D136" r:id="rId607"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H136" r:id="rId608"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV136" r:id="rId609"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C137" r:id="rId610"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D137" r:id="rId611"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H137" r:id="rId612"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV137" r:id="rId613"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C138" r:id="rId614"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D138" r:id="rId615"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H138" r:id="rId616"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV138" r:id="rId617"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C139" r:id="rId618"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D139" r:id="rId619"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H139" r:id="rId620"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV139" r:id="rId621"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C140" r:id="rId622"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D140" r:id="rId623"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H140" r:id="rId624"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV140" r:id="rId625"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C141" r:id="rId626"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D141" r:id="rId627"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H141" r:id="rId628"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV141" r:id="rId629"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C142" r:id="rId630"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D142" r:id="rId631"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H142" r:id="rId632"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV142" r:id="rId633"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C143" r:id="rId634"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D143" r:id="rId635"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H143" r:id="rId636"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV143" r:id="rId637"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C144" r:id="rId638"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D144" r:id="rId639"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H144" r:id="rId640"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV144" r:id="rId641"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C145" r:id="rId642"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D145" r:id="rId643"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H145" r:id="rId644"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV145" r:id="rId645"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C146" r:id="rId646"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D146" r:id="rId647"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H146" r:id="rId648"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV146" r:id="rId649"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C147" r:id="rId650"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D147" r:id="rId651"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H147" r:id="rId652"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV147" r:id="rId653"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C148" r:id="rId654"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D148" r:id="rId655"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H148" r:id="rId656"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV148" r:id="rId657"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C149" r:id="rId658"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D149" r:id="rId659"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H149" r:id="rId660"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV149" r:id="rId661"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C150" r:id="rId662"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D150" r:id="rId663"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H150" r:id="rId664"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV150" r:id="rId665"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C151" r:id="rId666"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D151" r:id="rId667"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H151" r:id="rId668"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV151" r:id="rId669"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C152" r:id="rId670"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D152" r:id="rId671"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H152" r:id="rId672"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV152" r:id="rId673"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C153" r:id="rId674"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D153" r:id="rId675"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H153" r:id="rId676"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV153" r:id="rId677"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C154" r:id="rId678"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D154" r:id="rId679"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H154" r:id="rId680"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV154" r:id="rId681"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C155" r:id="rId682"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D155" r:id="rId683"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H155" r:id="rId684"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV155" r:id="rId685"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C156" r:id="rId686"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D156" r:id="rId687"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H156" r:id="rId688"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV156" r:id="rId689"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C157" r:id="rId690"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D157" r:id="rId691"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H157" r:id="rId692"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV157" r:id="rId693"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C158" r:id="rId694"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D158" r:id="rId695"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H158" r:id="rId696"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV158" r:id="rId697"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C159" r:id="rId698"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D159" r:id="rId699"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H159" r:id="rId700"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV159" r:id="rId701"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C160" r:id="rId702"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D160" r:id="rId703"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H160" r:id="rId704"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV160" r:id="rId705"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C161" r:id="rId706"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D161" r:id="rId707"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H161" r:id="rId708"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV161" r:id="rId709"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C162" r:id="rId710"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D162" r:id="rId711"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H162" r:id="rId712"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV162" r:id="rId713"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C163" r:id="rId714"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D163" r:id="rId715"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H163" r:id="rId716"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV163" r:id="rId717"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C164" r:id="rId718"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D164" r:id="rId719"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H164" r:id="rId720"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV164" r:id="rId721"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C165" r:id="rId722"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D165" r:id="rId723"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H165" r:id="rId724"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV165" r:id="rId725"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C166" r:id="rId726"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D166" r:id="rId727"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H166" r:id="rId728"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV166" r:id="rId729"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C167" r:id="rId730"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D167" r:id="rId731"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H167" r:id="rId732"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV167" r:id="rId733"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C168" r:id="rId734"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D168" r:id="rId735"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H168" r:id="rId736"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV168" r:id="rId737"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C169" r:id="rId738"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D169" r:id="rId739"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H169" r:id="rId740"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV169" r:id="rId741"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C170" r:id="rId742"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D170" r:id="rId743"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H170" r:id="rId744"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV170" r:id="rId745"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C171" r:id="rId746"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D171" r:id="rId747"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H171" r:id="rId748"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV171" r:id="rId749"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C172" r:id="rId750"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D172" r:id="rId751"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H172" r:id="rId752"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV172" r:id="rId753"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C173" r:id="rId754"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D173" r:id="rId755"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H173" r:id="rId756"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV173" r:id="rId757"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C174" r:id="rId758"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D174" r:id="rId759"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H174" r:id="rId760"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV174" r:id="rId761"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C175" r:id="rId762"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D175" r:id="rId763"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H175" r:id="rId764"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV175" r:id="rId765"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C176" r:id="rId766"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D176" r:id="rId767"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H176" r:id="rId768"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV176" r:id="rId769"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C177" r:id="rId770"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D177" r:id="rId771"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H177" r:id="rId772"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV177" r:id="rId773"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>